<commit_message>
backup before fixing branch logic
</commit_message>
<xml_diff>
--- a/survey_results.xlsx
+++ b/survey_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,192 +424,290 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>LINE名</t>
+          <t>店舗名</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>手入力名</t>
+          <t>部門</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>名前</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Q5</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Q7理由</t>
-        </is>
-      </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ハラスメント</t>
+          <t>Q7</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>会社評価</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>会社への要望</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>組合への要望</t>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ハラスメント詳細</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>相談したか</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>結果</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>会社要望</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>組合要望</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-24 07:27:36</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>T_hashi</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>橋本</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>週2日休めている</t>
+          <t>2026-03-04 00:41:41</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>足りている</t>
+          <t>週２日休んでいる。</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>足りないので終業のタイムカードを打って仕事をしている。</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ほとんど毎日1時間</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>要員不足の為、仕方なく自らの判断で。</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>相談をした</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>話を聞いてくれない。</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>ない</t>
+          <t>テスト</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>できている</t>
+          <t>いいえ</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>公休すら休めないので取れない。</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ある</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>相談した</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>解決していない</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-24 07:42:06</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ごとう みき</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>ごとうみき</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>週2日休めている</t>
+          <t>2026-03-04 00:59:38</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>残業時間内で終わっている</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>6,その他</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+          <t>週２日休んでいる。</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>足りている。</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>はい</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>ない</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>できている</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-25 01:41:25</t>
+          <t>2026-03-04 02:03:35</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>久間木 剛</t>
+          <t>テスト</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>久間木　剛</t>
+          <t>テスト</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>週2日休めている</t>
+          <t>テスト</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>足りている</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+          <t>週１日しか休んでいない。もう1日はタイムカードを打刻せずにフルに出勤している。</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>足りないので終業のタイムカードを打って仕事をしている。</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ほとんど毎日１時間</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>要員不足の為、仕方なく自らの判断で。</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>相談をした</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>話を聞いてくれない。</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ない</t>
+          <t>テスト</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>できている</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+          <t>いいえ</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>公休すら休めないので取れない。</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ある</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>パワハラ</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>相談していない</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>解決していない</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>テスト</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>